<commit_message>
finished sprint backlog 3
</commit_message>
<xml_diff>
--- a/presentations/links/sprintbacklog3.xlsx
+++ b/presentations/links/sprintbacklog3.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="28810"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="18528"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yathanvidyananthan/Desktop/cscc01/L01_03/presentations/links/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yinli\Programming\CSCC01Repo\L01_03\presentations\links\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sprint Plan and Sprint Report" sheetId="5" r:id="rId1"/>
     <sheet name="Burndown Chart" sheetId="6" r:id="rId2"/>
     <sheet name="Taskboard Snapshots" sheetId="7" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="150001" concurrentCalc="0"/>
+  <calcPr calcId="171027" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
       <x14:workbookPr defaultImageDpi="32767"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="59">
   <si>
     <t>Task</t>
   </si>
@@ -115,13 +115,103 @@
     <t>As Bob Sponge (student), I need to be able to take a quiz for each lesson</t>
   </si>
   <si>
-    <t>As Sohee Kang (professor), I want each assignment/quiz to have randomized questions so that students don't have the same quiz</t>
+    <t>Create a backend call to create TA accounts</t>
+  </si>
+  <si>
+    <t>Create a backend call to create student accounts</t>
+  </si>
+  <si>
+    <t>Create a backend call to create assignments</t>
+  </si>
+  <si>
+    <t>Create a backend call to create questions</t>
+  </si>
+  <si>
+    <t>Create a backend call to edit questions</t>
+  </si>
+  <si>
+    <t>Get TA Account creation working with the backend</t>
+  </si>
+  <si>
+    <t>Get Student Account Creation working with the backend</t>
+  </si>
+  <si>
+    <t>Get assignment creation working with the backend</t>
+  </si>
+  <si>
+    <t>Create a backend call to list assignments</t>
+  </si>
+  <si>
+    <t>Get assignment list to pull data from the backend</t>
+  </si>
+  <si>
+    <t>Create a backend call to list questions</t>
+  </si>
+  <si>
+    <t>Create a page to edit questions from</t>
+  </si>
+  <si>
+    <t>Create a page for 10 questions</t>
+  </si>
+  <si>
+    <t>Create a template page that can be filled in for multiple choice</t>
+  </si>
+  <si>
+    <t>Create a template page for short answer</t>
+  </si>
+  <si>
+    <t>Create a backend call to return Question HTML</t>
+  </si>
+  <si>
+    <t>Create a Backend call to accept question responses</t>
+  </si>
+  <si>
+    <t>Linhai</t>
+  </si>
+  <si>
+    <t>t2</t>
+  </si>
+  <si>
+    <t>t1</t>
+  </si>
+  <si>
+    <t>t5</t>
+  </si>
+  <si>
+    <t>t6</t>
+  </si>
+  <si>
+    <t>t10</t>
+  </si>
+  <si>
+    <t>t11</t>
+  </si>
+  <si>
+    <t>Get login pages to poll the login backend</t>
+  </si>
+  <si>
+    <t>Jinming</t>
+  </si>
+  <si>
+    <t>shoaib</t>
+  </si>
+  <si>
+    <t>yathan</t>
+  </si>
+  <si>
+    <t>Yathan</t>
+  </si>
+  <si>
+    <t>Calvin</t>
+  </si>
+  <si>
+    <t>Shoaib</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -220,7 +310,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -237,12 +327,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -252,23 +336,24 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="27">
@@ -314,7 +399,7 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="en-US"/>
   <c:roundedCorners val="0"/>
@@ -358,7 +443,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -465,9 +549,8 @@
             <c:showPercent val="0"/>
             <c:showBubbleSize val="0"/>
             <c:showLeaderLines val="0"/>
-            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+            <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
                   <c:spPr>
@@ -492,28 +575,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.0</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.0</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.0</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.0</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.0</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -528,31 +611,31 @@
                   <c:v>18.5</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>16.0</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.0</c:v>
+                  <c:v>9</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>7.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>6.0</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>6.0</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.0</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>4.0</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000000-B8BC-4974-B628-0A342B1B0345}"/>
             </c:ext>
@@ -629,9 +712,8 @@
             <c:showPercent val="0"/>
             <c:showBubbleSize val="0"/>
             <c:showLeaderLines val="0"/>
-            <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+            <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
                 <c15:showLeaderLines val="1"/>
                 <c15:leaderLines>
                   <c:spPr>
@@ -656,28 +738,28 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="8"/>
                 <c:pt idx="0">
-                  <c:v>0.0</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1.0</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2.0</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.0</c:v>
+                  <c:v>3</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>4.0</c:v>
+                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>5.0</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>6.0</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>7.0</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -716,7 +798,7 @@
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
-          <c:extLst xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+          <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-B8BC-4974-B628-0A342B1B0345}"/>
             </c:ext>
@@ -769,7 +851,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -902,7 +983,6 @@
               </a:p>
             </c:rich>
           </c:tx>
-          <c:layout/>
           <c:overlay val="0"/>
           <c:spPr>
             <a:noFill/>
@@ -964,7 +1044,7 @@
           </a:p>
         </c:txPr>
         <c:crossAx val="1157409088"/>
-        <c:crossesAt val="1.0"/>
+        <c:crossesAt val="1"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
@@ -977,7 +1057,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="t"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:solidFill>
@@ -1693,7 +1772,7 @@
         <xdr:cNvPr id="3" name="Chart 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0100-000003000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0100-000003000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1998,30 +2077,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z29"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Z33"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="9.1640625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="53" style="4" customWidth="1"/>
     <col min="3" max="3" width="8" style="4" customWidth="1"/>
-    <col min="4" max="5" width="42.83203125" style="5" customWidth="1"/>
+    <col min="4" max="5" width="42.85546875" style="5" customWidth="1"/>
     <col min="6" max="6" width="14" style="5" customWidth="1"/>
-    <col min="7" max="7" width="8.33203125" style="1" customWidth="1"/>
-    <col min="8" max="8" width="2.83203125" style="3" customWidth="1"/>
-    <col min="9" max="9" width="13.5" style="1" customWidth="1"/>
-    <col min="10" max="10" width="14.5" style="12" customWidth="1"/>
-    <col min="11" max="11" width="5.83203125" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.28515625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="2.85546875" style="3" customWidth="1"/>
+    <col min="9" max="9" width="13.42578125" style="1" customWidth="1"/>
+    <col min="10" max="10" width="14.42578125" style="10" customWidth="1"/>
+    <col min="11" max="11" width="5.85546875" style="1" customWidth="1"/>
     <col min="12" max="13" width="6" style="1" bestFit="1" customWidth="1"/>
     <col min="14" max="16" width="6" style="1" customWidth="1"/>
     <col min="17" max="17" width="6" style="1" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="3.6640625" style="10" customWidth="1"/>
-    <col min="19" max="19" width="7" style="11" customWidth="1"/>
+    <col min="18" max="18" width="3.7109375" style="8" customWidth="1"/>
+    <col min="19" max="19" width="7" style="9" customWidth="1"/>
     <col min="20" max="26" width="6" style="1" customWidth="1"/>
     <col min="27" max="16384" width="12" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:26" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>4</v>
       </c>
@@ -2046,7 +2125,7 @@
       <c r="I1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="12" t="s">
+      <c r="J1" s="10" t="s">
         <v>13</v>
       </c>
       <c r="K1" s="3" t="s">
@@ -2070,7 +2149,7 @@
       <c r="Q1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="S1" s="11" t="s">
+      <c r="S1" s="9" t="s">
         <v>14</v>
       </c>
       <c r="T1" s="3" t="s">
@@ -2095,166 +2174,412 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="14">
+    <row r="2" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="16">
         <v>1</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="15" t="s">
         <v>11</v>
       </c>
       <c r="C2" s="4">
         <v>1</v>
       </c>
+      <c r="D2" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G2" s="1">
+        <v>3</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="N2" s="1">
+        <v>3</v>
+      </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A3" s="14"/>
-      <c r="B3" s="13"/>
-      <c r="C3" s="4">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="C3" s="5">
         <v>2</v>
       </c>
+      <c r="D3" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="1">
+        <v>1</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="P3" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A4" s="14"/>
-      <c r="B4" s="13"/>
-      <c r="C4" s="4">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A4" s="16"/>
+      <c r="B4" s="15"/>
+      <c r="C4" s="5">
         <v>3</v>
       </c>
+      <c r="D4" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="P4" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="5" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A5" s="14"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="4">
+    <row r="5" spans="1:26" ht="12" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="16"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="5">
         <v>4</v>
       </c>
+      <c r="D5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="1">
+        <v>3</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q5" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A6" s="14"/>
-      <c r="B6" s="13"/>
-      <c r="C6" s="4">
+    <row r="6" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A6" s="16"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="5">
         <v>5</v>
       </c>
+      <c r="D6" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="1">
+        <v>1</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Q6" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A7" s="14"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="4">
+    <row r="7" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A7" s="16">
+        <v>2</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="5">
         <v>6</v>
       </c>
+      <c r="D7" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="G7" s="1">
+        <v>1</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="N7" s="1">
+        <v>1</v>
+      </c>
+      <c r="P7" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="8" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A8" s="14"/>
-      <c r="B8" s="13"/>
-      <c r="C8" s="1">
+    <row r="8" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="16"/>
+      <c r="B8" s="17"/>
+      <c r="C8" s="5">
         <v>7</v>
       </c>
+      <c r="D8" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="G8" s="1">
+        <v>3</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="O8" s="1">
+        <v>3</v>
+      </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A9" s="14"/>
-      <c r="B9" s="13"/>
-      <c r="C9" s="1">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A9" s="16"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="5">
         <v>8</v>
       </c>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="H9" s="1"/>
+      <c r="D9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9" s="1">
+        <v>1</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="N9" s="1">
+        <v>1</v>
+      </c>
+      <c r="P9" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A10" s="14"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="1">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="C10" s="4">
         <v>9</v>
       </c>
+      <c r="D10" s="5" t="s">
+        <v>37</v>
+      </c>
       <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
+      <c r="F10" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1</v>
+      </c>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="O10" s="1">
+        <v>3</v>
+      </c>
     </row>
-    <row r="11" spans="1:26" ht="38.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A11" s="14"/>
-      <c r="B11" s="13"/>
-      <c r="C11" s="1">
+    <row r="11" spans="1:26" ht="38.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="14">
+        <v>3</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="4">
         <v>10</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
+      <c r="G11" s="1">
+        <v>1</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="P11" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="12" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A12" s="14">
-        <v>2</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>12</v>
-      </c>
+    <row r="12" spans="1:26" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="14"/>
+      <c r="B12" s="13"/>
       <c r="C12" s="5">
         <v>11</v>
       </c>
+      <c r="D12" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" s="1"/>
       <c r="F12" s="1"/>
+      <c r="G12" s="1">
+        <v>1</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="P12" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A13" s="14"/>
-      <c r="B13" s="15"/>
+    <row r="13" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
       <c r="C13" s="5">
         <v>12</v>
       </c>
-      <c r="F13" s="1"/>
+      <c r="D13" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="G13" s="1">
+        <v>3</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="P13" s="1">
+        <v>3</v>
+      </c>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A14" s="14"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="5">
+    <row r="14" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="C14" s="4">
         <v>13</v>
       </c>
+      <c r="D14" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" s="1">
+        <v>2</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="P14" s="1">
+        <v>2</v>
+      </c>
     </row>
-    <row r="15" spans="1:26" ht="51" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="9">
-        <v>3</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>16</v>
+    <row r="15" spans="1:26" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="14">
+        <v>4</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>26</v>
       </c>
       <c r="C15" s="5">
         <v>14</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>18</v>
+        <v>32</v>
+      </c>
+      <c r="G15" s="1">
+        <v>1</v>
+      </c>
+      <c r="I15" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A16" s="9"/>
-      <c r="B16" s="8"/>
+    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A16" s="14"/>
+      <c r="B16" s="5"/>
       <c r="C16" s="5">
         <v>15</v>
       </c>
       <c r="D16" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="G16" s="1">
+        <v>2</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="P16" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:26" ht="26.1" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="14">
+        <v>5</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="5">
+        <v>16</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G17" s="1">
+        <v>1</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="M17" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A18" s="14"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="5">
         <v>17</v>
       </c>
+      <c r="D18" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G18" s="1">
+        <v>1</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M18" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="17" spans="1:26" ht="26" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A17" s="9">
-        <v>4</v>
-      </c>
-      <c r="B17" s="18" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A18" s="9"/>
-      <c r="B18" s="18"/>
-    </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A19" s="9"/>
-      <c r="B19" s="18"/>
-      <c r="G19" s="2"/>
+    <row r="19" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A19" s="14"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5">
+        <v>18</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G19" s="1">
+        <v>2</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>45</v>
+      </c>
       <c r="K19" s="2"/>
       <c r="L19" s="2"/>
       <c r="M19" s="2"/>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
-      <c r="P19" s="2"/>
+      <c r="P19" s="1">
+        <v>2</v>
+      </c>
       <c r="Q19" s="2"/>
       <c r="Z19" s="2"/>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A20" s="9"/>
-      <c r="B20" s="18"/>
+    <row r="20" spans="1:26" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A20" s="14"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="5">
+        <v>19</v>
+      </c>
+      <c r="D20" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="G20" s="1">
+        <v>2</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="P20" s="1">
+        <v>2</v>
+      </c>
       <c r="T20" s="2"/>
       <c r="U20" s="2"/>
       <c r="V20" s="2"/>
@@ -2262,67 +2587,67 @@
       <c r="X20" s="2"/>
       <c r="Y20" s="2"/>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A21" s="9"/>
-      <c r="B21" s="18"/>
+    <row r="21" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="C21" s="5">
+        <v>20</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="G21" s="1">
+        <v>1</v>
+      </c>
+      <c r="I21" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M21" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="22" spans="1:26" ht="26" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A22" s="9">
+    <row r="22" spans="1:26" ht="26.1" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="24" spans="1:26" ht="15" x14ac:dyDescent="0.25">
+      <c r="G24" s="2">
+        <f>SUM(G2:G23)</f>
+        <v>32</v>
+      </c>
+      <c r="K24" s="6">
+        <f>SUM(K2:K22)</f>
+        <v>0</v>
+      </c>
+      <c r="L24" s="6">
+        <f t="shared" ref="L24:Q24" si="0">SUM(L2:L22)</f>
+        <v>0</v>
+      </c>
+      <c r="M24" s="6">
+        <f t="shared" si="0"/>
+        <v>3</v>
+      </c>
+      <c r="N24" s="6">
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="B22" s="18" t="s">
-        <v>27</v>
+      <c r="O24" s="6">
+        <f t="shared" si="0"/>
+        <v>6</v>
+      </c>
+      <c r="P24" s="6">
+        <f t="shared" si="0"/>
+        <v>17</v>
+      </c>
+      <c r="Q24" s="6">
+        <f t="shared" si="0"/>
+        <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A23" s="9"/>
-      <c r="B23" s="18"/>
-    </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A24" s="9"/>
-      <c r="B24" s="18"/>
-    </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A25" s="9"/>
-      <c r="B25" s="18"/>
-    </row>
-    <row r="26" spans="1:26" ht="15" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A26" s="9">
-        <v>6</v>
-      </c>
-      <c r="B26" s="18" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A27" s="9"/>
-      <c r="B27" s="18"/>
-    </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A28" s="9"/>
-      <c r="B28" s="18"/>
-    </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.15">
-      <c r="A29" s="9"/>
-      <c r="B29" s="18"/>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="14"/>
+      <c r="B33" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="15">
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="A15:A16"/>
+  <mergeCells count="3">
     <mergeCell ref="R1:R1048576"/>
     <mergeCell ref="S1:S1048576"/>
     <mergeCell ref="J1:J1048576"/>
-    <mergeCell ref="B2:B11"/>
-    <mergeCell ref="A2:A11"/>
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="A12:A14"/>
-    <mergeCell ref="B17:B21"/>
-    <mergeCell ref="A17:A21"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="A22:A25"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="A26:A29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -2330,30 +2655,30 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="3" width="4.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" customWidth="1"/>
+    <col min="2" max="3" width="4.85546875" customWidth="1"/>
     <col min="4" max="4" width="5" customWidth="1"/>
-    <col min="5" max="9" width="4.83203125" customWidth="1"/>
+    <col min="5" max="9" width="4.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
-      <c r="F1" s="16"/>
-      <c r="G1" s="16"/>
-      <c r="H1" s="16"/>
-      <c r="I1" s="16"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>10</v>
       </c>
@@ -2382,7 +2707,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>8</v>
       </c>
@@ -2411,7 +2736,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>7</v>
       </c>
@@ -2440,16 +2765,16 @@
         <v>18.5</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A5" s="17"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="12"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
+      <c r="I5" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2463,9 +2788,9 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2480,7 +2805,56 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?><ct:contentTypeSchema ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F770ABC8F9B27C4C8461F4575C23FAEA" ma:contentTypeVersion="1" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6f0f4afd6cc55b40f57cb0d59e49aa45" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes">
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10001</Type>
+    <SequenceNumber>1000</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10002</Type>
+    <SequenceNumber>1001</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10004</Type>
+    <SequenceNumber>1002</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+  <Receiver>
+    <Name>Document ID Generator</Name>
+    <Synchronization>Synchronous</Synchronization>
+    <Type>10006</Type>
+    <SequenceNumber>1003</SequenceNumber>
+    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
+    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
+    <Data/>
+    <Filter/>
+  </Receiver>
+</spe:Receivers>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?><p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"><documentManagement><_dlc_DocId xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07">WORK-769-153</_dlc_DocId><_dlc_DocIdUrl xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07"><Url>http://intranet/workingtogether/projects/110405/_layouts/DocIdRedir.aspx?ID=WORK-769-153</Url><Description>WORK-769-153</Description></_dlc_DocIdUrl><IconOverlay xmlns="http://schemas.microsoft.com/sharepoint/v4" xsi:nil="true"/><Last_x0020_Archive xmlns="$ListId:Shared Documents;" xsi:nil="true"/><Reason xmlns="$ListId:Shared Documents;" xsi:nil="true"></Reason></documentManagement></p:properties>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?><ct:contentTypeSchema ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F770ABC8F9B27C4C8461F4575C23FAEA" ma:contentTypeVersion="1" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6f0f4afd6cc55b40f57cb0d59e49aa45" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes">
 <xsd:schema targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0f7c28edf12e174e47f2c7bd2736e8bd" ns2:_="" ns3:_="" ns4:_="" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0d93dc7d-5998-434b-bf34-aa89b432ec07" xmlns:ns3="$ListId:Shared Documents;" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v4">
 <xsd:import namespace="0d93dc7d-5998-434b-bf34-aa89b432ec07"/>
 <xsd:import namespace="$ListId:Shared Documents;"/>
@@ -2654,55 +3028,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?><p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"><documentManagement><_dlc_DocId xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07">WORK-769-153</_dlc_DocId><_dlc_DocIdUrl xmlns="0d93dc7d-5998-434b-bf34-aa89b432ec07"><Url>http://intranet/workingtogether/projects/110405/_layouts/DocIdRedir.aspx?ID=WORK-769-153</Url><Description>WORK-769-153</Description></_dlc_DocIdUrl><IconOverlay xmlns="http://schemas.microsoft.com/sharepoint/v4" xsi:nil="true"/><Last_x0020_Archive xmlns="$ListId:Shared Documents;" xsi:nil="true"/><Reason xmlns="$ListId:Shared Documents;" xsi:nil="true"></Reason></documentManagement></p:properties>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10001</Type>
-    <SequenceNumber>1000</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10002</Type>
-    <SequenceNumber>1001</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10004</Type>
-    <SequenceNumber>1002</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-  <Receiver>
-    <Name>Document ID Generator</Name>
-    <Synchronization>Synchronous</Synchronization>
-    <Type>10006</Type>
-    <SequenceNumber>1003</SequenceNumber>
-    <Assembly>Microsoft.Office.DocumentManagement, Version=14.0.0.0, Culture=neutral, PublicKeyToken=71e9bce111e9429c</Assembly>
-    <Class>Microsoft.Office.DocumentManagement.Internal.DocIdHandler</Class>
-    <Data/>
-    <Filter/>
-  </Receiver>
-</spe:Receivers>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D2B9EEEF-7393-4E57-9716-D967A23AC816}">
   <ds:schemaRefs>
@@ -2712,6 +3037,26 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F807D2B-FCE5-4B63-BC9A-551BEF173D66}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47BCCC64-3980-40D2-8C4F-F5BACE67ECB4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="0d93dc7d-5998-434b-bf34-aa89b432ec07"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v4"/>
+    <ds:schemaRef ds:uri="$ListId:Shared Documents;"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0008E140-BD0E-4C41-947D-F18B1A1E4B6B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2729,24 +3074,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47BCCC64-3980-40D2-8C4F-F5BACE67ECB4}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="0d93dc7d-5998-434b-bf34-aa89b432ec07"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v4"/>
-    <ds:schemaRef ds:uri="$ListId:Shared Documents;"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F807D2B-FCE5-4B63-BC9A-551BEF173D66}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/events"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>